<commit_message>
Stage 8 WIP: fix rounds in progress
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UWExrN7wNZ4prKGqMsXc4Z
</commit_message>
<xml_diff>
--- a/public/downloads/engine-workshop-solution.xlsx
+++ b/public/downloads/engine-workshop-solution.xlsx
@@ -12088,6 +12088,35 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="7">
+    <dataValidation sqref="B18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="ערך לא תקין" error="הון עצמי נוסף: מספר בין 0 ל־500,000" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>500000</formula2>
+    </dataValidation>
+    <dataValidation sqref="B19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="ערך לא תקין" error="0 (לא) או 1 (כן)" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation sqref="B20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="ערך לא תקין" error="0 (לא) או 1 (כן)" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation sqref="B21" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="ערך לא תקין" error="בנק: a, b, c או d" type="list">
+      <formula1>"a,b,c,d"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="ערך לא תקין" error="משקולת: מספר שלם בין 0 ל־100" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation sqref="B23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="ערך לא תקין" error="משקולת: מספר שלם בין 0 ל־100" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation sqref="B24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="ערך לא תקין" error="משקולת: מספר שלם בין 0 ל־100" type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12176,7 +12205,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="str">
-        <f>IF(ISNUMBER(D5),IF(ABS(D5)&lt;=E5,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D5),IF(ABS(D5)&lt;=E5,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12201,7 +12230,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="str">
-        <f>IF(ISNUMBER(D6),IF(ABS(D6)&lt;=E6,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D6),IF(ABS(D6)&lt;=E6,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12226,7 +12255,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="str">
-        <f>IF(ISNUMBER(D7),IF(ABS(D7)&lt;=E7,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D7),IF(ABS(D7)&lt;=E7,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12272,7 +12301,7 @@
         <v>0.05</v>
       </c>
       <c r="F9" t="str">
-        <f>IF(ISNUMBER(D9),IF(ABS(D9)&lt;=E9,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D9),IF(ABS(D9)&lt;=E9,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12297,7 +12326,7 @@
         <v>6</v>
       </c>
       <c r="F10" t="str">
-        <f>IF(ISNUMBER(D10),IF(ABS(D10)&lt;=E10,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D10),IF(ABS(D10)&lt;=E10,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12312,17 +12341,17 @@
         <v>1030.73179174652</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>1031.61</v>
+        <v>1030.73</v>
       </c>
       <c r="D11" s="10">
         <f>IF(ISNUMBER(B11),B11-C11,"")</f>
-        <v>-0.878208253475577</v>
+        <v>0.00179174652430447</v>
       </c>
       <c r="E11" t="n">
         <v>10</v>
       </c>
       <c r="F11" t="str">
-        <f>IF(ISNUMBER(D11),IF(ABS(D11)&lt;=E11,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D11),IF(ABS(D11)&lt;=E11,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12347,7 +12376,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="str">
-        <f>IF(ISNUMBER(D12),IF(ABS(D12)&lt;=E12,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D12),IF(ABS(D12)&lt;=E12,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12372,7 +12401,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="str">
-        <f>IF(ISNUMBER(D13),IF(ABS(D13)&lt;=E13,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D13),IF(ABS(D13)&lt;=E13,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12397,7 +12426,7 @@
         <v>0</v>
       </c>
       <c r="F14" t="str">
-        <f>IF(ISNUMBER(D14),IF(ABS(D14)&lt;=E14,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D14),IF(ABS(D14)&lt;=E14,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12422,7 +12451,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="str">
-        <f>IF(ISNUMBER(D15),IF(ABS(D15)&lt;=E15,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D15),IF(ABS(D15)&lt;=E15,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12447,7 +12476,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="str">
-        <f>IF(ISNUMBER(D16),IF(ABS(D16)&lt;=E16,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D16),IF(ABS(D16)&lt;=E16,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12472,7 +12501,7 @@
         <v>0</v>
       </c>
       <c r="F17" t="str">
-        <f>IF(ISNUMBER(D17),IF(ABS(D17)&lt;=E17,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D17),IF(ABS(D17)&lt;=E17,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12497,7 +12526,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="str">
-        <f>IF(ISNUMBER(D18),IF(ABS(D18)&lt;=E18,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D18),IF(ABS(D18)&lt;=E18,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12522,7 +12551,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="str">
-        <f>IF(ISNUMBER(D19),IF(ABS(D19)&lt;=E19,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D19),IF(ABS(D19)&lt;=E19,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12547,7 +12576,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="str">
-        <f>IF(ISNUMBER(D20),IF(ABS(D20)&lt;=E20,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D20),IF(ABS(D20)&lt;=E20,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12572,7 +12601,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="str">
-        <f>IF(ISNUMBER(D21),IF(ABS(D21)&lt;=E21,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D21),IF(ABS(D21)&lt;=E21,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12597,7 +12626,7 @@
         <v>0.05</v>
       </c>
       <c r="F22" t="str">
-        <f>IF(ISNUMBER(D22),IF(ABS(D22)&lt;=E22,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D22),IF(ABS(D22)&lt;=E22,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12622,7 +12651,7 @@
         <v>6</v>
       </c>
       <c r="F23" t="str">
-        <f>IF(ISNUMBER(D23),IF(ABS(D23)&lt;=E23,"✓","✗"),"")</f>
+        <f>IF(ISNUMBER(D23),IF(ABS(D23)&lt;=E23,"✓","✗"),"✗")</f>
         <v>✓</v>
       </c>
     </row>
@@ -12650,7 +12679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -12687,7 +12716,7 @@
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>1 — מיצוב: בתאים B18 עד B21 בחרו הון עצמי נוסף, סגירת הלוואת הרכב, הורה וכנס. ההלוואה, שיעור המימון והכנסה הפנויה מתעדכנים (שורות 45 עד 56).</t>
+          <t>1 — מיצוב: בתאים B18 עד B21 בחרו הון עצמי נוסף, סגירת הלוואת הרכב, הורה ובנק. ההלוואה, שיעור המימון והכנסה הפנויה מתעדכנים (שורות 45 עד 56).</t>
         </is>
       </c>
     </row>
@@ -12701,7 +12730,7 @@
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>3 — חיפוש: הרשת היא כל התמהילים בצעדים של 10 אחוזים (66). אין להוסיף שורות: מרחב החיפוש הוא מה שנבדק.</t>
+          <t>3 — חיפוש: הרשת היא כל התמהילים בצעדים של 10 אחוזים (66). אין להוסיף שורות: מרחב החיפוש הוא מה שנבדק. שורת הרשת הראשונה (89) מלאה בכל העמודות כדוגמה. עמדו על כותרת של עמודה כדי לקרוא מה היא עושה (בכותרות עם הערה), העתיקו את השורה למטה עד שורה 154, ובדקו שהתוצאות בשורות 59 עד 69 התמלאו.</t>
         </is>
       </c>
     </row>
@@ -12736,40 +12765,47 @@
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
         <is>
-          <t>8 — בדיקה מול הצעת בנק: בתאים E4 עד F18 יש הצעה לדוגמה של בנק בדוי. האומדן הוא המחירון של הבנק; ההצעה היא מה שהוא כתב. הפער נמדד בהחזר הראשון ובסך התשלומים.</t>
+          <t>8 — בדיקה מול הצעת בנק: בתאים E4 עד F11 יש הצעה לדוגמה של בנק בדוי. האומדן הוא המחירון של הבנק; ההצעה היא מה שהוא כתב. הפער נמדד בהחזר הראשון ובסך התשלומים.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>התאים F13 עד F18 מלאים: אומדן, הצעה והפער בהחזר הראשון ובסך התשלומים.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>הלשונית ״בדיקה״</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="23" t="inlineStr">
-        <is>
-          <t>היא משווה את הגיליון למנוע של הקורס לקלט ההתחלתי. הסבילות היא כמה שקלים, כי הגיליון לא מעגל כל ריבית חודשית.</t>
-        </is>
-      </c>
-    </row>
     <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>היא משווה את הגיליון למנוע של הקורס לקלט ההתחלתי. הסבילות היא כמה שקלים, כי הגיליון לא מעגל כל ריבית חודשית. בתבנית היא מתעדכנת בזמן שאתם ממלאים: עמודה C היא התוצאות של המנוע, כך שאפשר להציץ בה בסוף, וכשהכול מתאים יופיע ✓ בתחתית.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>Excel ו־Google Sheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="23" t="inlineStr">
-        <is>
-          <t>בחלק מההגדרות האזוריות מפרידים בין ארגומנטים בנקודה־פסיק (;). הגיליון משתמש בפונקציות PMT, SUMPRODUCT, COUNTIFS ו־INDEX: הכול קיים גם ב־Google Sheets.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>בחלק מההגדרות האזוריות מפרידים בין ארגומנטים בנקודה־פסיק (;). הגיליון משתמש בפונקציות PMT, SUMPRODUCT, COUNTIFS ו־INDEX: הכול קיים גם ב־Google Sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>שינוי בחירה ישנה את התוצאות, וגם את הבדיקה: היא נכונה לקלט ההתחלתי בלבד.</t>
         </is>

</xml_diff>

<commit_message>
Stage 8: fixes 8.22-8.28 (D), engine projected maximum
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UWExrN7wNZ4prKGqMsXc4Z
</commit_message>
<xml_diff>
--- a/public/downloads/engine-workshop-solution.xlsx
+++ b/public/downloads/engine-workshop-solution.xlsx
@@ -12348,7 +12348,7 @@
         <v>0.00179174652430447</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>0.05</v>
       </c>
       <c r="F11" t="str">
         <f>IF(ISNUMBER(D11),IF(ABS(D11)&lt;=E11,"✓","✗"),"✗")</f>
@@ -12658,7 +12658,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>הגיליון מקרב את המנוע: הוא מחשב החזר מדויק (בלי עיגול כל ריבית חודשית), והמנוע מעגל כל חודש לאגורה. בסך התשלומים הפער עד כמה שקלים. בחשיפה הפער עד כעשרה שקלים, כי במנוע התשלום האחרון סוגר את היתרה, והוא גבוה בכמה שקלים מהתשלום הקבוע. הבחירה של התמהיל לא מושפעת.</t>
+          <t>הגיליון מקרב את המנוע: הוא מחשב החזר מדויק (בלי עיגול כל ריבית חודשית), והמנוע מעגל כל חודש לאגורה. בסך התשלומים הפער עד כמה שקלים, כי במנוע התשלום האחרון סוגר את היתרה והוא שונה בכמה שקלים מהקבוע. בחשיפה אין פער של ממש, כי המנוע לא סופר את התשלום האחרון בהחזר הגבוה. הבחירה של התמהיל לא מושפעת.</t>
         </is>
       </c>
     </row>

</xml_diff>